<commit_message>
Reframe UC1 as an out-of-fold back-test and add end-to-end recording guide
The brief is now dated 1 Oct 2026 (after the Jul-Sep outcome window) and the
target list is a back-test scored with out-of-fold predictions, so no
customer is scored by a model that trained on them. Task notes, metadata,
use-case doc and Use_Cases_v2.xlsx updated to match. New
UC1_Recording_Guide_Windows_Teams.md covers setup, rehearsal, Teams
recording, the minute-by-minute take with reference numbers, and review.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/use_cases/Use_Cases_v2.xlsx
+++ b/use_cases/Use_Cases_v2.xlsx
@@ -558,11 +558,11 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Use case: A retail bank wants to predict which existing customers are likely to buy another product in the next 90 days. You build a model, validate it, explain what drives the next purchase, and use it to pick the Q3 campaign target list.
-Goal: Develop, validate and explain a cross-sell model, then package it and produce a budget- and compliance-constrained target list.
-Starting material (synthetic data only): input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, cross-sell label ~11.6%, CRM duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.docx (budget 4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints).
-Approach: Read brief &amp; dictionary &gt; explore data and fix quality issues &gt; leakage audit &gt; stratified train/test split &gt; logistic baseline &gt; gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; score &amp; build target list &gt; package with README.
-Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data and fix quality issues. 3) Remove leaky/protected fields and make a leak-free stratified split. 4) Train a baseline and make improvements. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Score customers, apply compliance rules, select top 4,000 and validate ROI in Excel. 8) Package model with a README, reproduce results, 3-slide summary.</t>
+          <t>Use case: A retail bank wants to predict which existing customers are likely to buy another product in the next 90 days. You build a model, validate it, explain what drives the next purchase, and prove its value with an out-of-sample back-test of the campaign target list.
+Goal: Develop, validate and explain a cross-sell model, then package it and back-test a budget- and compliance-constrained target list against actual outcomes.
+Starting material (synthetic data only): input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, CRM duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.docx (budget 4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints).
+Approach: Read brief &amp; dictionary &gt; explore data and fix quality issues &gt; leakage audit &gt; stratified train/test split &gt; logistic baseline &gt; gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; out-of-fold back-test of the target list &gt; package with README.
+Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data and fix quality issues. 3) Remove leaky/protected fields and make a leak-free stratified split. 4) Train a baseline and make improvements. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Score customers out of fold, apply compliance rules, select top 4,000 and compare expected vs actual conversions and ROI with random selection in Excel. 8) Package model with a README, reproduce results, 3-slide summary.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -583,8 +583,8 @@
       <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Problem statement : Cross-selling products to the existing customer base improves revenue, but random campaigns waste most of the budget (only ~1 in 9 customers convert) and most companies have not identified which existing customers are most likely to buy another product.
-Solution : This video demonstrates how a senior data scientist builds and explains a cross-sell model using Microsoft Word, Microsoft Excel, Visual Studio Code (Jupyter) and Microsoft PowerPoint - catching leaky fields, handling class imbalance, checking calibration, and turning the model into a compliant, budget-sized target list. The output will be: Notebook; Q3 target list with ROI (Excel); model package with README; 3-slide summary.
-How the result is checked: Metrics on a hold-out the model has not seen (ROC-AUC &gt;= 0.78, top-20% lift &gt;= 2.5x); no leakage and no gender used; baseline is beaten on PR-AUC or the reason is explained; target list has exactly 4,000 compliant rows; metrics reproduce on re-run.
+Solution : This video demonstrates how a senior data scientist builds and explains a cross-sell model using Microsoft Word, Microsoft Excel, Visual Studio Code (Jupyter) and Microsoft PowerPoint - catching leaky fields, handling class imbalance, checking calibration, and proving the value with an out-of-sample back-test of a compliant, budget-sized target list. The output will be: Notebook; back-test target list with ROI (Excel); model package with README; 3-slide summary.
+How the result is checked: Metrics on a hold-out the model has not seen (ROC-AUC &gt;= 0.78, top-20% lift &gt;= 2.5x); no leakage and no gender used; baseline is beaten on PR-AUC or the reason is explained; back-test list has exactly 4,000 compliant rows converting at &gt;= 2x the eligible average; metrics reproduce on re-run.
 Estimated recording length: ~35 minutes.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
UC1: pre-written team pipeline with planted fixes, Excel pivots, deck template
Following the internal benchmark recording, UC1 now ships the team's
existing pipeline (pipeline_config.py + notebooks 01-04) under
Deliverables/1_Input, 2_Code, 3_Intermediate, 4_Output. Five realistic
issues (date format and label drift, missing imputer, leaky new column,
labels-vs-probabilities evaluation) are fixed on camera; selftest_uc1.py
proves each fails and each fix works. Adds an Excel pivot EDA segment, a
PowerPoint template (input 4), the answer key, and rewrites the recording
guide, use-case doc, task notes, metadata and Use_Cases_v2.xlsx.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/use_cases/Use_Cases_v2.xlsx
+++ b/use_cases/Use_Cases_v2.xlsx
@@ -558,16 +558,16 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Use case: A retail bank wants to predict which existing customers are likely to buy another product in the next 90 days. You build a model, validate it, explain what drives the next purchase, and prove its value with an out-of-sample back-test of the campaign target list.
+          <t>Use case: A retail bank wants to predict which existing customers are likely to buy another product in the next 90 days. You run and fix the team's existing cross-sell pipeline on a new data extract, validate and explain the model, and prove its value with an out-of-sample back-test of the campaign target list.
 Goal: Develop, validate and explain a cross-sell model, then package it and back-test a budget- and compliance-constrained target list against actual outcomes.
-Starting material (synthetic data only): input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, CRM duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.docx (budget 4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints).
-Approach: Read brief &amp; dictionary &gt; explore data and fix quality issues &gt; leakage audit &gt; stratified train/test split &gt; logistic baseline &gt; gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; out-of-fold back-test of the target list &gt; package with README.
-Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data and fix quality issues. 3) Remove leaky/protected fields and make a leak-free stratified split. 4) Train a baseline and make improvements. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Score customers out of fold, apply compliance rules, select top 4,000 and compare expected vs actual conversions and ROI with random selection in Excel. 8) Package model with a README, reproduce results, 3-slide summary.</t>
+Starting material (synthetic data only): input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.docx (4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, back-test) built for an earlier snapshot.
+Approach: Read brief &amp; dictionary &gt; explore the raw data with Excel PivotTables &gt; run the pipeline on the new extract and fix what breaks (date formats, label drift, missing imputer, leaky new column, evaluation bug) &gt; stratified split, logistic baseline vs gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; out-of-fold back-test &gt; package with README &gt; validate ROI in Excel &gt; summary deck.
+Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data in Excel pivots (drivers, data quality, leakage, missingness). 3) Run preprocessing and fix data-quality / schema-drift issues. 4) Run training: leak-free stratified split, baseline vs improved model, fix the leakage. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Back-test the 4,000-customer list out of fold and compare expected vs actual conversions and ROI with random selection in Excel. 8) Package model with a README and complete the summary deck.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Microsoft Word, Microsoft Excel, Visual Studio Code (Jupyter + Python: pandas, scikit-learn, SHAP), Microsoft PowerPoint, Finder</t>
+          <t>Microsoft Word, Microsoft Excel (PivotTables, formulas), Visual Studio Code (Jupyter + Python: pandas, scikit-learn, SHAP), Microsoft PowerPoint, Finder</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -577,20 +577,20 @@
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>2-3 hours (estimated for a ~35-minute video)</t>
+          <t>2-3 hours (estimated for a ~38-minute video)</t>
         </is>
       </c>
       <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Problem statement : Cross-selling products to the existing customer base improves revenue, but random campaigns waste most of the budget (only ~1 in 9 customers convert) and most companies have not identified which existing customers are most likely to buy another product.
-Solution : This video demonstrates how a senior data scientist builds and explains a cross-sell model using Microsoft Word, Microsoft Excel, Visual Studio Code (Jupyter) and Microsoft PowerPoint - catching leaky fields, handling class imbalance, checking calibration, and proving the value with an out-of-sample back-test of a compliant, budget-sized target list. The output will be: Notebook; back-test target list with ROI (Excel); model package with README; 3-slide summary.
-How the result is checked: Metrics on a hold-out the model has not seen (ROC-AUC &gt;= 0.78, top-20% lift &gt;= 2.5x); no leakage and no gender used; baseline is beaten on PR-AUC or the reason is explained; back-test list has exactly 4,000 compliant rows converting at &gt;= 2x the eligible average; metrics reproduce on re-run.
-Estimated recording length: ~35 minutes.</t>
+Solution : This video demonstrates how a senior data scientist explores the data in Microsoft Excel, runs and debugs the team's existing cross-sell pipeline in Visual Studio Code (Jupyter) on a changed data extract - catching schema drift, a leaky new column and an evaluation bug - validates and explains the model, and proves the value with an out-of-sample back-test, finishing the summary in Microsoft PowerPoint. The output will be: Pivot analysis; corrected pipeline and model package with README; back-test target list with ROI (Excel); summary deck.
+How the result is checked: Metrics on a hold-out the model has not seen (ROC-AUC &gt;= 0.78, top-20% lift &gt;= 2.5x); no leakage and no gender used; baseline is beaten on PR-AUC or the reason is explained; back-test list has exactly 4,000 compliant rows scored out of fold and converting at &gt;= 2x the eligible average.
+Estimated recording length: ~38 minutes.</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera); added Word (brief) and Excel (data dictionary, target list) so 3+ apps form a connected workflow; added stakeholder brief with constraints and acceptance criteria; added leakage, compliance and budget/ROI checks to show expert judgment (Mercor intern test).</t>
+          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the team's pre-existing pipeline (documented as a pre-existing asset) that is run, debugged and interpreted on camera, as in the internal benchmark. Added Excel pivot exploration and ROI validation, Word brief and a PowerPoint template so 3+ apps form a connected workflow; added leakage, compliance and an out-of-fold back-test with ROI to show expert judgment.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add single UC1 recording script; remove data-origin wording
UC1_RECORDING_SCRIPT.md replaces the separate recording guide: setup,
rehearsal, Teams, and a scene-by-scene take with clicks, narration, all
five code fixes, expected outputs and a numbers cheat sheet. Removes
data-origin wording from the deck template footer, Metadata.rtf,
Use_Cases_v2.xlsx, use-case docs, generators and README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/use_cases/Use_Cases_v2.xlsx
+++ b/use_cases/Use_Cases_v2.xlsx
@@ -560,7 +560,7 @@
         <is>
           <t>Use case: A retail bank wants to predict which existing customers are likely to buy another product in the next 90 days. You run and fix the team's existing cross-sell pipeline on a new data extract, validate and explain the model, and prove its value with an out-of-sample back-test of the campaign target list.
 Goal: Develop, validate and explain a cross-sell model, then package it and back-test a budget- and compliance-constrained target list against actual outcomes.
-Starting material (synthetic data only): input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.docx (4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, back-test) built for an earlier snapshot.
+Starting material: input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.docx (4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, back-test) built for an earlier snapshot.
 Approach: Read brief &amp; dictionary &gt; explore the raw data with Excel PivotTables &gt; run the pipeline on the new extract and fix what breaks (date formats, label drift, missing imputer, leaky new column, evaluation bug) &gt; stratified split, logistic baseline vs gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; out-of-fold back-test &gt; package with README &gt; validate ROI in Excel &gt; summary deck.
 Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data in Excel pivots (drivers, data quality, leakage, missingness). 3) Run preprocessing and fix data-quality / schema-drift issues. 4) Run training: leak-free stratified split, baseline vs improved model, fix the leakage. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Back-test the 4,000-customer list out of fold and compare expected vs actual conversions and ROI with random selection in Excel. 8) Package model with a README and complete the summary deck.</t>
         </is>
@@ -624,7 +624,7 @@
         <is>
           <t>Use case: A lender wants to predict which customers in early collections are likely to pay within 30 days. An ML model is built, validated out of time, calibrated, and used to prioritise agent effort; the drivers of payment are explained.
 Goal: Develop, validate and explain a propensity-to-pay model, then package it and produce a capacity-constrained agent work list.
-Starting material (synthetic data only): input 1 - collections accounts.csv (20,000 accounts entering collections Jan-Jun 2026 with paid/not-paid label, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - collections strategy brief.docx (25 agents / ~37% capacity, day-7 scoring point, calibration, dispute &amp; hardship exclusions).
+Starting material: input 1 - collections accounts.csv (20,000 accounts entering collections Jan-Jun 2026 with paid/not-paid label, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - collections strategy brief.docx (25 agents / ~37% capacity, day-7 scoring point, calibration, dispute &amp; hardship exclusions).
 Approach: Read brief &amp; dictionary &gt; explore data and fix quality issues &gt; leakage audit against the day-7 decision point &gt; out-of-time split (train Jan-Apr, calibrate May, test June) &gt; business-rule and logistic baselines &gt; gradient boosting &gt; calibrate &gt; explain drivers (SHAP) &gt; build work list &gt; package with README.
 Steps to narrate: 1) Review brief and data dictionary, flag fields captured after day 7. 2) Explore the data and fix quality issues (mixed date formats, business-rule violations). 3) Make a leak-free out-of-time split and show the drift. 4) Train baselines and make improvements. 5) Evaluate with the right metrics and check/correct calibration. 6) Explain the drivers of the outcome. 7) Rank June accounts by expected unpaid amount within capacity and validate in Excel. 8) Package model with a README, reproduce results, 3-slide summary.</t>
         </is>

</xml_diff>

<commit_message>
Deliverable-rule packager; UC2 rebuilt as pre-written pipeline with script
- prep/package_deliverables (.py/.cmd/.sh): after a take, validates labels,
  required files, planted-bug fixes and notebook errors, then builds
  Deliverables.zip with the original code as input 5 and the corrected code
  as final output 4 (no __pycache__ or other junk)
- UC2: inputs moved to 1_Input; team pipeline (config + 4 notebooks) with five
  bugs distinct from UC1; selftest_uc2.py; deck template; answer key;
  UC2_RECORDING_SCRIPT.md; Metadata, task notes, use-case doc and
  Use_Cases_v2.xlsx updated. Data generator strengthened so boosting beats
  the baseline (planted data issues unchanged)
- Deck templates built by one generator; UC1 script and Metadata mention the
  packager and input 5 / final output 4

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/use_cases/Use_Cases_v2.xlsx
+++ b/use_cases/Use_Cases_v2.xlsx
@@ -622,16 +622,16 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Use case: A lender wants to predict which customers in early collections are likely to pay within 30 days. An ML model is built, validated out of time, calibrated, and used to prioritise agent effort; the drivers of payment are explained.
-Goal: Develop, validate and explain a propensity-to-pay model, then package it and produce a capacity-constrained agent work list.
-Starting material: input 1 - collections accounts.csv (20,000 accounts entering collections Jan-Jun 2026 with paid/not-paid label, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - collections strategy brief.docx (25 agents / ~37% capacity, day-7 scoring point, calibration, dispute &amp; hardship exclusions).
-Approach: Read brief &amp; dictionary &gt; explore data and fix quality issues &gt; leakage audit against the day-7 decision point &gt; out-of-time split (train Jan-Apr, calibrate May, test June) &gt; business-rule and logistic baselines &gt; gradient boosting &gt; calibrate &gt; explain drivers (SHAP) &gt; build work list &gt; package with README.
-Steps to narrate: 1) Review brief and data dictionary, flag fields captured after day 7. 2) Explore the data and fix quality issues (mixed date formats, business-rule violations). 3) Make a leak-free out-of-time split and show the drift. 4) Train baselines and make improvements. 5) Evaluate with the right metrics and check/correct calibration. 6) Explain the drivers of the outcome. 7) Rank June accounts by expected unpaid amount within capacity and validate in Excel. 8) Package model with a README, reproduce results, 3-slide summary.</t>
+          <t>Use case: A lender wants to predict which customers in early collections are likely to pay within 30 days. You run and fix the team's existing propensity-to-pay pipeline on a new collections extract, validate it out of time, calibrate it, explain what drives payment, and use it to prioritise agent effort.
+Goal: Develop, validate and explain a propensity-to-pay model, then package it and produce a capacity-constrained June agent work list.
+Starting material: input 1 - collections accounts.csv (20,000 accounts entering collections Jan-Jun 2026 with paid/not-paid label, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - collections strategy brief.docx (25 agents / ~37% capacity, day-7 scoring point, calibration, dispute &amp; hardship exclusions); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, work list) built for last year's extract.
+Approach: Read brief &amp; dictionary &gt; explore the raw data with Excel PivotTables &gt; run the pipeline and fix what breaks (date misparse, zero incomes, time-window overlap, post-day-7 leak, inverted expected-loss ranking) &gt; out-of-time split (train Jan-Apr, calibrate May, test June) &gt; business-rule and logistic baselines vs gradient boosting &gt; calibrate &gt; explain drivers (SHAP) &gt; build work list &gt; package with README &gt; validate in Excel &gt; summary deck.
+Steps to narrate: 1) Review brief and data dictionary, flag fields captured after day 7. 2) Explore the data in Excel pivots (products, employment, leakage, payment history). 3) Run preprocessing and fix data-quality issues (mixed date formats, zero incomes, business-rule violations). 4) Make a leak-free out-of-time split, show the drift, fix the leakage. 5) Evaluate on June with the right metrics and check/correct calibration. 6) Explain the drivers of the outcome. 7) Rank June accounts by expected unpaid amount within capacity, compare with today's rule and validate in Excel. 8) Package model with a README and complete the summary deck.</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Microsoft Word, Microsoft Excel, Visual Studio Code (Jupyter + Python: pandas, scikit-learn, SHAP), Microsoft PowerPoint, Finder</t>
+          <t>Microsoft Word, Microsoft Excel (PivotTables, formulas), Visual Studio Code (Jupyter + Python: pandas, scikit-learn, SHAP), Microsoft PowerPoint, Finder</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -641,20 +641,20 @@
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>2-3 hours (estimated for a ~35-minute video)</t>
+          <t>2-3 hours (estimated for a ~38-minute video)</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Problem statement : Improving collections is important to meet the monthly targets, but cure rates are falling and agents call the most overdue accounts first; the customers with the highest likelihood of needing an agent - weighted by amount owed - have to be identified to maximise collections.
-Solution : This video demonstrates how a senior data scientist builds and explains a propensity-to-pay model using Microsoft Word, Microsoft Excel, Visual Studio Code (Jupyter) and Microsoft PowerPoint - validating out of time to expose drift, recalibrating probabilities, and producing an agent work list that beats the current rule. The output will be: Notebook; June agent work list (Excel); model package with README; 3-slide summary.
-How the result is checked: Out-of-time metrics on months the model has not seen (ROC-AUC &gt;= 0.78); no leakage (nothing captured after day 7); baselines (current DPD rule and logistic regression) are beaten or the reason is explained; calibration checked and corrected; work list fits capacity; metrics reproduce on re-run.
-Estimated recording length: ~35 minutes.</t>
+Solution : This video demonstrates how a senior data scientist explores the data in Microsoft Excel, runs and debugs the team's existing propensity-to-pay pipeline in Visual Studio Code (Jupyter) - catching a silent date misparse, a time-window overlap, a post-decision leak and an inverted ranking - validates out of time, recalibrates the probabilities and produces an agent work list that beats the current rule, finishing the summary in Microsoft PowerPoint. The output will be: Pivot analysis; corrected pipeline and model package with README; validated June agent work list (Excel); summary deck.
+How the result is checked: Out-of-time metrics on a month the model has not seen (ROC-AUC &gt;= 0.78); no leakage (nothing captured after day 7); baselines (current DPD rule and logistic regression) are beaten or the reason is explained; calibration checked and corrected; work list fits capacity.
+Estimated recording length: ~38 minutes.</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera); added Word and Excel; switched to out-of-time validation with calibration, day-7 leakage rule, business-rule baseline and capacity-constrained work list - clearly different from UC1 so it is not rejected as a duplicate.</t>
+          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the team's pre-existing pipeline (documented as a pre-existing asset) that is run, debugged and interpreted on camera, as in the internal benchmark. Added Excel pivots and validation, Word brief and PowerPoint template; out-of-time validation with calibration, day-7 leakage rule, business-rule baseline and capacity-constrained work list - clearly different from UC1 so it is not rejected as a duplicate.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch on-camera apps to what the Mac has: VS Code, Firefox, LibreOffice
The provided Mac has no Microsoft Office. Task notes become Task Notes.md
shown as a VS Code Markdown preview (staging opens .md files in preview and
hides Metadata.rtf); briefs are generated as PDF and read in Firefox;
pivots and validation move to LibreOffice Calc and the deck to LibreOffice
Impress. Both recording scripts, Metadata topology, use-case docs,
Use_Cases_v2.xlsx, WINDOWS_SETUP, the Mac checklist, verifier and packager
updated; Q1 resolved. UC1 deck template rebuilt with the new chart name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/use_cases/Use_Cases_v2.xlsx
+++ b/use_cases/Use_Cases_v2.xlsx
@@ -560,14 +560,14 @@
         <is>
           <t>Use case: A retail bank wants to predict which existing customers are likely to buy another product in the next 90 days. You run and fix the team's existing cross-sell pipeline on a new data extract, validate and explain the model, and prove its value with an out-of-sample back-test of the campaign target list.
 Goal: Develop, validate and explain a cross-sell model, then package it and back-test a budget- and compliance-constrained target list against actual outcomes.
-Starting material: input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.docx (4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, back-test) built for an earlier snapshot.
-Approach: Read brief &amp; dictionary &gt; explore the raw data with Excel PivotTables &gt; run the pipeline on the new extract and fix what breaks (date formats, label drift, missing imputer, leaky new column, evaluation bug) &gt; stratified split, logistic baseline vs gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; out-of-fold back-test &gt; package with README &gt; validate ROI in Excel &gt; summary deck.
-Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data in Excel pivots (drivers, data quality, leakage, missingness). 3) Run preprocessing and fix data-quality / schema-drift issues. 4) Run training: leak-free stratified split, baseline vs improved model, fix the leakage. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Back-test the 4,000-customer list out of fold and compare expected vs actual conversions and ROI with random selection in Excel. 8) Package model with a README and complete the summary deck.</t>
+Starting material: input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.pdf (4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, back-test) built for an earlier snapshot.
+Approach: Read brief &amp; dictionary &gt; explore the raw data with LibreOffice Calc pivot tables &gt; run the pipeline on the new extract and fix what breaks (date formats, label drift, missing imputer, leaky new column, evaluation bug) &gt; stratified split, logistic baseline vs gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; out-of-fold back-test &gt; package with README &gt; validate ROI in LibreOffice Calc &gt; summary deck.
+Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data in LibreOffice Calc pivots (drivers, data quality, leakage, missingness). 3) Run preprocessing and fix data-quality / schema-drift issues. 4) Run training: leak-free stratified split, baseline vs improved model, fix the leakage. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Back-test the 4,000-customer list out of fold and compare expected vs actual conversions and ROI with random selection in LibreOffice Calc. 8) Package model with a README and complete the summary deck.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Microsoft Word, Microsoft Excel (PivotTables, formulas), Visual Studio Code (Jupyter + Python: pandas, scikit-learn, SHAP), Microsoft PowerPoint, Finder</t>
+          <t>Firefox (PDF brief), LibreOffice Calc (pivot tables, formulas), Visual Studio Code (Markdown preview, Jupyter + Python: pandas, scikit-learn, SHAP), LibreOffice Impress, Finder</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -583,14 +583,14 @@
       <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Problem statement : Cross-selling products to the existing customer base improves revenue, but random campaigns waste most of the budget (only ~1 in 9 customers convert) and most companies have not identified which existing customers are most likely to buy another product.
-Solution : This video demonstrates how a senior data scientist explores the data in Microsoft Excel, runs and debugs the team's existing cross-sell pipeline in Visual Studio Code (Jupyter) on a changed data extract - catching schema drift, a leaky new column and an evaluation bug - validates and explains the model, and proves the value with an out-of-sample back-test, finishing the summary in Microsoft PowerPoint. The output will be: Pivot analysis; corrected pipeline and model package with README; back-test target list with ROI (Excel); summary deck.
+Solution : This video demonstrates how a senior data scientist explores the data in LibreOffice Calc, runs and debugs the team's existing cross-sell pipeline in Visual Studio Code (Jupyter) on a changed data extract - catching schema drift, a leaky new column and an evaluation bug - validates and explains the model, and proves the value with an out-of-sample back-test, finishing the summary in LibreOffice Impress. The output will be: Pivot analysis; corrected pipeline and model package with README; back-test target list with ROI (LibreOffice Calc); summary deck.
 How the result is checked: Metrics on a hold-out the model has not seen (ROC-AUC &gt;= 0.78, top-20% lift &gt;= 2.5x); no leakage and no gender used; baseline is beaten on PR-AUC or the reason is explained; back-test list has exactly 4,000 compliant rows scored out of fold and converting at &gt;= 2x the eligible average.
 Estimated recording length: ~38 minutes.</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the team's pre-existing pipeline (documented as a pre-existing asset) that is run, debugged and interpreted on camera, as in the internal benchmark. Added Excel pivot exploration and ROI validation, Word brief and a PowerPoint template so 3+ apps form a connected workflow; added leakage, compliance and an out-of-fold back-test with ROI to show expert judgment.</t>
+          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the team's pre-existing pipeline (documented as a pre-existing asset) that is run, debugged and interpreted on camera, as in the internal benchmark. Added LibreOffice Calc pivot exploration and ROI validation, a PDF brief in Firefox and an Impress deck template (no Microsoft Office on the Mac) so 3+ apps form a connected workflow; added leakage, compliance and an out-of-fold back-test with ROI to show expert judgment.</t>
         </is>
       </c>
     </row>
@@ -624,14 +624,14 @@
         <is>
           <t>Use case: A lender wants to predict which customers in early collections are likely to pay within 30 days. You run and fix the team's existing propensity-to-pay pipeline on a new collections extract, validate it out of time, calibrate it, explain what drives payment, and use it to prioritise agent effort.
 Goal: Develop, validate and explain a propensity-to-pay model, then package it and produce a capacity-constrained June agent work list.
-Starting material: input 1 - collections accounts.csv (20,000 accounts entering collections Jan-Jun 2026 with paid/not-paid label, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - collections strategy brief.docx (25 agents / ~37% capacity, day-7 scoring point, calibration, dispute &amp; hardship exclusions); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, work list) built for last year's extract.
-Approach: Read brief &amp; dictionary &gt; explore the raw data with Excel PivotTables &gt; run the pipeline and fix what breaks (date misparse, zero incomes, time-window overlap, post-day-7 leak, inverted expected-loss ranking) &gt; out-of-time split (train Jan-Apr, calibrate May, test June) &gt; business-rule and logistic baselines vs gradient boosting &gt; calibrate &gt; explain drivers (SHAP) &gt; build work list &gt; package with README &gt; validate in Excel &gt; summary deck.
-Steps to narrate: 1) Review brief and data dictionary, flag fields captured after day 7. 2) Explore the data in Excel pivots (products, employment, leakage, payment history). 3) Run preprocessing and fix data-quality issues (mixed date formats, zero incomes, business-rule violations). 4) Make a leak-free out-of-time split, show the drift, fix the leakage. 5) Evaluate on June with the right metrics and check/correct calibration. 6) Explain the drivers of the outcome. 7) Rank June accounts by expected unpaid amount within capacity, compare with today's rule and validate in Excel. 8) Package model with a README and complete the summary deck.</t>
+Starting material: input 1 - collections accounts.csv (20,000 accounts entering collections Jan-Jun 2026 with paid/not-paid label, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - collections strategy brief.pdf (25 agents / ~37% capacity, day-7 scoring point, calibration, dispute &amp; hardship exclusions); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, work list) built for last year's extract.
+Approach: Read brief &amp; dictionary &gt; explore the raw data with LibreOffice Calc pivot tables &gt; run the pipeline and fix what breaks (date misparse, zero incomes, time-window overlap, post-day-7 leak, inverted expected-loss ranking) &gt; out-of-time split (train Jan-Apr, calibrate May, test June) &gt; business-rule and logistic baselines vs gradient boosting &gt; calibrate &gt; explain drivers (SHAP) &gt; build work list &gt; package with README &gt; validate in LibreOffice Calc &gt; summary deck.
+Steps to narrate: 1) Review brief and data dictionary, flag fields captured after day 7. 2) Explore the data in LibreOffice Calc pivots (products, employment, leakage, payment history). 3) Run preprocessing and fix data-quality issues (mixed date formats, zero incomes, business-rule violations). 4) Make a leak-free out-of-time split, show the drift, fix the leakage. 5) Evaluate on June with the right metrics and check/correct calibration. 6) Explain the drivers of the outcome. 7) Rank June accounts by expected unpaid amount within capacity, compare with today's rule and validate in LibreOffice Calc. 8) Package model with a README and complete the summary deck.</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Microsoft Word, Microsoft Excel (PivotTables, formulas), Visual Studio Code (Jupyter + Python: pandas, scikit-learn, SHAP), Microsoft PowerPoint, Finder</t>
+          <t>Firefox (PDF brief), LibreOffice Calc (pivot tables, formulas), Visual Studio Code (Markdown preview, Jupyter + Python: pandas, scikit-learn, SHAP), LibreOffice Impress, Finder</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -647,14 +647,14 @@
       <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Problem statement : Improving collections is important to meet the monthly targets, but cure rates are falling and agents call the most overdue accounts first; the customers with the highest likelihood of needing an agent - weighted by amount owed - have to be identified to maximise collections.
-Solution : This video demonstrates how a senior data scientist explores the data in Microsoft Excel, runs and debugs the team's existing propensity-to-pay pipeline in Visual Studio Code (Jupyter) - catching a silent date misparse, a time-window overlap, a post-decision leak and an inverted ranking - validates out of time, recalibrates the probabilities and produces an agent work list that beats the current rule, finishing the summary in Microsoft PowerPoint. The output will be: Pivot analysis; corrected pipeline and model package with README; validated June agent work list (Excel); summary deck.
+Solution : This video demonstrates how a senior data scientist explores the data in LibreOffice Calc, runs and debugs the team's existing propensity-to-pay pipeline in Visual Studio Code (Jupyter) - catching a silent date misparse, a time-window overlap, a post-decision leak and an inverted ranking - validates out of time, recalibrates the probabilities and produces an agent work list that beats the current rule, finishing the summary in LibreOffice Impress. The output will be: Pivot analysis; corrected pipeline and model package with README; validated June agent work list (LibreOffice Calc); summary deck.
 How the result is checked: Out-of-time metrics on a month the model has not seen (ROC-AUC &gt;= 0.78); no leakage (nothing captured after day 7); baselines (current DPD rule and logistic regression) are beaten or the reason is explained; calibration checked and corrected; work list fits capacity.
 Estimated recording length: ~38 minutes.</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the team's pre-existing pipeline (documented as a pre-existing asset) that is run, debugged and interpreted on camera, as in the internal benchmark. Added Excel pivots and validation, Word brief and PowerPoint template; out-of-time validation with calibration, day-7 leakage rule, business-rule baseline and capacity-constrained work list - clearly different from UC1 so it is not rejected as a duplicate.</t>
+          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the team's pre-existing pipeline (documented as a pre-existing asset) that is run, debugged and interpreted on camera, as in the internal benchmark. Added LibreOffice Calc pivots and validation, PDF brief in Firefox and an Impress deck template; out-of-time validation with calibration, day-7 leakage rule, business-rule baseline and capacity-constrained work list - clearly different from UC1 so it is not rejected as a duplicate.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Change story to: I built this pipeline and walk through its first full run
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/use_cases/Use_Cases_v2.xlsx
+++ b/use_cases/Use_Cases_v2.xlsx
@@ -558,11 +558,11 @@
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Use case: A retail bank wants to predict which existing customers are likely to buy another product in the next 90 days. You run and fix the team's existing cross-sell pipeline on a new data extract, validate and explain the model, and prove its value with an out-of-sample back-test of the campaign target list.
+          <t>Use case: A retail bank wants to predict which existing customers are likely to buy another product in the next 90 days. You walk through, run and fix the cross-sell pipeline you built for this request, validate and explain the model, and prove its value with an out-of-sample back-test of the campaign target list.
 Goal: Develop, validate and explain a cross-sell model, then package it and back-test a budget- and compliance-constrained target list against actual outcomes.
-Starting material: input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.pdf (4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, back-test) built for an earlier snapshot.
-Approach: Read brief &amp; dictionary &gt; explore the raw data with LibreOffice Calc pivot tables &gt; run the pipeline on the new extract and fix what breaks (date formats, label drift, missing imputer, leaky new column, evaluation bug) &gt; stratified split, logistic baseline vs gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; out-of-fold back-test &gt; package with README &gt; validate ROI in LibreOffice Calc &gt; summary deck.
-Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data in LibreOffice Calc pivots (drivers, data quality, leakage, missingness). 3) Run preprocessing and fix data-quality / schema-drift issues. 4) Run training: leak-free stratified split, baseline vs improved model, fix the leakage. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Back-test the 4,000-customer list out of fold and compare expected vs actual conversions and ROI with random selection in LibreOffice Calc. 8) Package model with a README and complete the summary deck.</t>
+Starting material: input 1 - customers.csv (20,000 customers, 30-Jun-2026 snapshot, Jul-Sep cross-sell label ~11.6%, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - campaign brief.pdf (4,000 contacts, $4/contact, $150 margin, opt-in only, no gender, exclude 2+ complaints); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, back-test) built for this request.
+Approach: Read brief &amp; dictionary &gt; explore the raw data with LibreOffice Calc pivot tables &gt; run the pipeline end to end and fix what the first full run exposes (date formats, label drift, missing imputer, leaky column, evaluation bug) &gt; stratified split, logistic baseline vs gradient boosting &gt; validate (PR-AUC, lift, calibration) &gt; explain drivers (SHAP) &gt; out-of-fold back-test &gt; package with README &gt; validate ROI in LibreOffice Calc &gt; summary deck.
+Steps to narrate: 1) Review brief and data dictionary, flag leakage suspects. 2) Explore the data in LibreOffice Calc pivots (drivers, data quality, leakage, missingness). 3) Run preprocessing and fix data-quality issues. 4) Run training: leak-free stratified split, baseline vs improved model, fix the leakage. 5) Evaluate with the right metric for the imbalance (PR-AUC, decile lift, calibration). 6) Explain the drivers of the outcome. 7) Back-test the 4,000-customer list out of fold and compare expected vs actual conversions and ROI with random selection in LibreOffice Calc. 8) Package model with a README and complete the summary deck.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
@@ -583,14 +583,14 @@
       <c r="J2" s="7" t="inlineStr">
         <is>
           <t>Problem statement : Cross-selling products to the existing customer base improves revenue, but random campaigns waste most of the budget (only ~1 in 9 customers convert) and most companies have not identified which existing customers are most likely to buy another product.
-Solution : This video demonstrates how a senior data scientist explores the data in LibreOffice Calc, runs and debugs the team's existing cross-sell pipeline in Visual Studio Code (Jupyter) on a changed data extract - catching schema drift, a leaky new column and an evaluation bug - validates and explains the model, and proves the value with an out-of-sample back-test, finishing the summary in LibreOffice Impress. The output will be: Pivot analysis; corrected pipeline and model package with README; back-test target list with ROI (LibreOffice Calc); summary deck.
+Solution : This video demonstrates how a senior data scientist explores the data in LibreOffice Calc, walks through, runs and debugs their own cross-sell pipeline in Visual Studio Code (Jupyter) - catching data-quality breaks, a leaky column and an evaluation bug - validates and explains the model, and proves the value with an out-of-sample back-test, finishing the summary in LibreOffice Impress. The output will be: Pivot analysis; corrected pipeline and model package with README; back-test target list with ROI (LibreOffice Calc); summary deck.
 How the result is checked: Metrics on a hold-out the model has not seen (ROC-AUC &gt;= 0.78, top-20% lift &gt;= 2.5x); no leakage and no gender used; baseline is beaten on PR-AUC or the reason is explained; back-test list has exactly 4,000 compliant rows scored out of fold and converting at &gt;= 2x the eligible average.
 Estimated recording length: ~38 minutes.</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the team's pre-existing pipeline (documented as a pre-existing asset) that is run, debugged and interpreted on camera, as in the internal benchmark. Added LibreOffice Calc pivot exploration and ROI validation, a PDF brief in Firefox and an Impress deck template (no Microsoft Office on the Mac) so 3+ apps form a connected workflow; added leakage, compliance and an out-of-fold back-test with ROI to show expert judgment.</t>
+          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the expert's own pipeline, prepared for this request (documented as a pre-existing asset), that is walked through, run, debugged and interpreted on camera, as in the internal benchmark. Added LibreOffice Calc pivot exploration and ROI validation, a PDF brief in Firefox and an Impress deck template (no Microsoft Office on the Mac) so 3+ apps form a connected workflow; added leakage, compliance and an out-of-fold back-test with ROI to show expert judgment.</t>
         </is>
       </c>
     </row>
@@ -622,10 +622,10 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Use case: A lender wants to predict which customers in early collections are likely to pay within 30 days. You run and fix the team's existing propensity-to-pay pipeline on a new collections extract, validate it out of time, calibrate it, explain what drives payment, and use it to prioritise agent effort.
+          <t>Use case: A lender wants to predict which customers in early collections are likely to pay within 30 days. You walk through, run and fix the propensity-to-pay pipeline you built for this request, validate it out of time, calibrate it, explain what drives payment, and use it to prioritise agent effort.
 Goal: Develop, validate and explain a propensity-to-pay model, then package it and produce a capacity-constrained June agent work list.
-Starting material: input 1 - collections accounts.csv (20,000 accounts entering collections Jan-Jun 2026 with paid/not-paid label, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - collections strategy brief.pdf (25 agents / ~37% capacity, day-7 scoring point, calibration, dispute &amp; hardship exclusions); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, work list) built for last year's extract.
-Approach: Read brief &amp; dictionary &gt; explore the raw data with LibreOffice Calc pivot tables &gt; run the pipeline and fix what breaks (date misparse, zero incomes, time-window overlap, post-day-7 leak, inverted expected-loss ranking) &gt; out-of-time split (train Jan-Apr, calibrate May, test June) &gt; business-rule and logistic baselines vs gradient boosting &gt; calibrate &gt; explain drivers (SHAP) &gt; build work list &gt; package with README &gt; validate in LibreOffice Calc &gt; summary deck.
+Starting material: input 1 - collections accounts.csv (20,000 accounts entering collections Jan-Jun 2026 with paid/not-paid label, duplicates and quality issues); input 2 - data dictionary.xlsx; input 3 - collections strategy brief.pdf (25 agents / ~37% capacity, day-7 scoring point, calibration, dispute &amp; hardship exclusions); input 4 - summary deck template.pptx; pre-existing pipeline code (config + 4 notebooks: preprocessing, training, testing, work list) built for this request.
+Approach: Read brief &amp; dictionary &gt; explore the raw data with LibreOffice Calc pivot tables &gt; run the pipeline end to end and fix what the first full run exposes (date misparse, zero incomes, time-window overlap, post-day-7 leak, inverted expected-loss ranking) &gt; out-of-time split (train Jan-Apr, calibrate May, test June) &gt; business-rule and logistic baselines vs gradient boosting &gt; calibrate &gt; explain drivers (SHAP) &gt; build work list &gt; package with README &gt; validate in LibreOffice Calc &gt; summary deck.
 Steps to narrate: 1) Review brief and data dictionary, flag fields captured after day 7. 2) Explore the data in LibreOffice Calc pivots (products, employment, leakage, payment history). 3) Run preprocessing and fix data-quality issues (mixed date formats, zero incomes, business-rule violations). 4) Make a leak-free out-of-time split, show the drift, fix the leakage. 5) Evaluate on June with the right metrics and check/correct calibration. 6) Explain the drivers of the outcome. 7) Rank June accounts by expected unpaid amount within capacity, compare with today's rule and validate in LibreOffice Calc. 8) Package model with a README and complete the summary deck.</t>
         </is>
       </c>
@@ -647,14 +647,14 @@
       <c r="J3" s="7" t="inlineStr">
         <is>
           <t>Problem statement : Improving collections is important to meet the monthly targets, but cure rates are falling and agents call the most overdue accounts first; the customers with the highest likelihood of needing an agent - weighted by amount owed - have to be identified to maximise collections.
-Solution : This video demonstrates how a senior data scientist explores the data in LibreOffice Calc, runs and debugs the team's existing propensity-to-pay pipeline in Visual Studio Code (Jupyter) - catching a silent date misparse, a time-window overlap, a post-decision leak and an inverted ranking - validates out of time, recalibrates the probabilities and produces an agent work list that beats the current rule, finishing the summary in LibreOffice Impress. The output will be: Pivot analysis; corrected pipeline and model package with README; validated June agent work list (LibreOffice Calc); summary deck.
+Solution : This video demonstrates how a senior data scientist explores the data in LibreOffice Calc, walks through, runs and debugs their own propensity-to-pay pipeline in Visual Studio Code (Jupyter) - catching a silent date misparse, a time-window overlap, a post-decision leak and an inverted ranking - validates out of time, recalibrates the probabilities and produces an agent work list that beats the current rule, finishing the summary in LibreOffice Impress. The output will be: Pivot analysis; corrected pipeline and model package with README; validated June agent work list (LibreOffice Calc); summary deck.
 How the result is checked: Out-of-time metrics on a month the model has not seen (ROC-AUC &gt;= 0.78); no leakage (nothing captured after day 7); baselines (current DPD rule and logistic regression) are beaten or the reason is explained; calibration checked and corrected; work list fits capacity.
 Estimated recording length: ~38 minutes.</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
-          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the team's pre-existing pipeline (documented as a pre-existing asset) that is run, debugged and interpreted on camera, as in the internal benchmark. Added LibreOffice Calc pivots and validation, PDF brief in Firefox and an Impress deck template; out-of-time validation with calibration, day-7 leakage rule, business-rule baseline and capacity-constrained work list - clearly different from UC1 so it is not rejected as a duplicate.</t>
+          <t>Use case unchanged. Removed Internal AutoML Tool, Terminal and GitHub Desktop (no Git on camera). Code is the expert's own pipeline, prepared for this request (documented as a pre-existing asset), that is walked through, run, debugged and interpreted on camera, as in the internal benchmark. Added LibreOffice Calc pivots and validation, PDF brief in Firefox and an Impress deck template; out-of-time validation with calibration, day-7 leakage rule, business-rule baseline and capacity-constrained work list - clearly different from UC1 so it is not rejected as a duplicate.</t>
         </is>
       </c>
     </row>

</xml_diff>